<commit_message>
Made sulfate-reducing bacteria decomposers in RhynieGuildStructure, renamed "std" to "sd" in web_metrics.jl
</commit_message>
<xml_diff>
--- a/data/rhynie/RhynieGuildStructure.xlsx
+++ b/data/rhynie/RhynieGuildStructure.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tannerfrank/Dropbox/Work/Devonian terr ecosystems/EcolNetworks/RhynieWebRepo/data/rhynie/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A7A4759-46E8-1544-A674-DD159484C60F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E46136AB-C9BD-DA42-A8C1-B31ABECBBA34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="28800" windowHeight="16580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3379,7 +3379,7 @@
         <v>9</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>9</v>
+        <v>78</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>

</xml_diff>